<commit_message>
update data and formats
</commit_message>
<xml_diff>
--- a/teams/benefits-portfolio/benefits-intake-optimization-pingwind/post-go-live/21-4140/21-4140-post-go-live-submission-tracker.xlsx
+++ b/teams/benefits-portfolio/benefits-intake-optimization-pingwind/post-go-live/21-4140/21-4140-post-go-live-submission-tracker.xlsx
@@ -84,6 +84,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -105,12 +106,14 @@
       <color theme="3"/>
       <name val="Aptos Display"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -118,6 +121,7 @@
       <color theme="3"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -169,20 +173,30 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -210,7 +224,7 @@
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF4EFB34"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -248,14 +262,14 @@
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF46B1E1"/>
+      <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF0E2841"/>
+      <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
@@ -382,91 +396,91 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="37.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.92"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <f aca="false">B4/B3</f>
+        <v>0.00166666666666667</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="0" t="n">
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="3" t="e">
-        <f aca="false">B4/B3</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>